<commit_message>
Add visitor counter full photo gallery and founders
</commit_message>
<xml_diff>
--- a/docs/downloads/苗栗文學作家資料庫.xlsx
+++ b/docs/downloads/苗栗文學作家資料庫.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="R063c349fd86a4385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作家資料庫" sheetId="2" r:id="R95db46a3d5fa43de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="R26b36db7cee44cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作家資料庫" sheetId="2" r:id="Rd71b452902284e76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -793,8 +793,7 @@
         <x:v>外部來源連結</x:v>
       </x:c>
       <x:c r="E8" s="33" t="n">
-        <x:f>COUNTA('作家資料庫'!$N$2:$N$40)+COUNTA('作家資料庫'!$P$2:$P$40)+COUNTA('作家資料庫'!$R$2:$R$40)</x:f>
-        <x:v>117</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
         <x:v>逐筆列於資料表的來源網址欄</x:v>
@@ -3158,7 +3157,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48f59d3723f44f16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra471b8d0fced4367"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add trail map news and gallery navigation refinements
</commit_message>
<xml_diff>
--- a/docs/downloads/苗栗文學作家資料庫.xlsx
+++ b/docs/downloads/苗栗文學作家資料庫.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="R26b36db7cee44cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作家資料庫" sheetId="2" r:id="Rd71b452902284e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="R6241b4e198214a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作家資料庫" sheetId="2" r:id="Raefde2e8f5f546c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1350,7 +1350,7 @@
         <x:v>古典文學</x:v>
       </x:c>
       <x:c r="C9" s="86" t="str">
-        <x:v>陳瑚（字滄玉）</x:v>
+        <x:v>陳瑚</x:v>
       </x:c>
       <x:c r="D9" s="86" t="str">
         <x:v>1875—1922</x:v>
@@ -3157,7 +3157,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra471b8d0fced4367"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6ef11270b494beb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>